<commit_message>
Removed unnecessary functions and modules for contamination assessment work of Chapter 2.
</commit_message>
<xml_diff>
--- a/results/ref_threshold_sensitivity/tables/MaxRel_rda_axes_summary.xlsx
+++ b/results/ref_threshold_sensitivity/tables/MaxRel_rda_axes_summary.xlsx
@@ -475,16 +475,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3.51</v>
+        <v>5.42</v>
       </c>
       <c r="D2" t="n">
-        <v>61.77</v>
+        <v>74.55</v>
       </c>
       <c r="E2" t="n">
-        <v>61.77</v>
+        <v>74.55</v>
       </c>
       <c r="F2" t="n">
-        <v>7.01</v>
+        <v>13.7</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -505,19 +505,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.89</v>
+        <v>1.03</v>
       </c>
       <c r="D3" t="n">
-        <v>15.75</v>
+        <v>14.13</v>
       </c>
       <c r="E3" t="n">
-        <v>77.52</v>
+        <v>88.68000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>1.79</v>
+        <v>2.6</v>
       </c>
       <c r="G3" t="n">
-        <v>0.77</v>
+        <v>0.47</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -535,19 +535,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.61</v>
+        <v>0.54</v>
       </c>
       <c r="D4" t="n">
-        <v>10.73</v>
+        <v>7.41</v>
       </c>
       <c r="E4" t="n">
-        <v>88.25</v>
+        <v>96.09</v>
       </c>
       <c r="F4" t="n">
-        <v>1.22</v>
+        <v>1.36</v>
       </c>
       <c r="G4" t="n">
-        <v>0.97</v>
+        <v>0.93</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -565,16 +565,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.39</v>
+        <v>0.16</v>
       </c>
       <c r="D5" t="n">
-        <v>6.91</v>
+        <v>2.27</v>
       </c>
       <c r="E5" t="n">
-        <v>95.16</v>
+        <v>98.36</v>
       </c>
       <c r="F5" t="n">
-        <v>0.78</v>
+        <v>0.42</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -595,16 +595,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.28</v>
+        <v>0.12</v>
       </c>
       <c r="D6" t="n">
-        <v>4.84</v>
+        <v>1.64</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>0.55</v>
+        <v>0.3</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Added MRT to take over the taxa clustering analysis, refactored the stage 1 and 2 modules. Comparisons between MRT and WardsLDA are made.
</commit_message>
<xml_diff>
--- a/results/ref_threshold_sensitivity/tables/MaxRel_rda_axes_summary.xlsx
+++ b/results/ref_threshold_sensitivity/tables/MaxRel_rda_axes_summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -475,23 +475,23 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5.42</v>
+        <v>1.42</v>
       </c>
       <c r="D2" t="n">
-        <v>74.55</v>
+        <v>53.13</v>
       </c>
       <c r="E2" t="n">
-        <v>74.55</v>
+        <v>53.13</v>
       </c>
       <c r="F2" t="n">
-        <v>13.7</v>
+        <v>4.3</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>**</t>
+          <t>*</t>
         </is>
       </c>
     </row>
@@ -505,19 +505,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.03</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>14.13</v>
+        <v>20.71</v>
       </c>
       <c r="E3" t="n">
-        <v>88.68000000000001</v>
+        <v>73.83</v>
       </c>
       <c r="F3" t="n">
-        <v>2.6</v>
+        <v>1.67</v>
       </c>
       <c r="G3" t="n">
-        <v>0.47</v>
+        <v>0.84</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -535,19 +535,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.54</v>
+        <v>0.38</v>
       </c>
       <c r="D4" t="n">
-        <v>7.41</v>
+        <v>14.22</v>
       </c>
       <c r="E4" t="n">
-        <v>96.09</v>
+        <v>88.06</v>
       </c>
       <c r="F4" t="n">
-        <v>1.36</v>
+        <v>1.15</v>
       </c>
       <c r="G4" t="n">
-        <v>0.93</v>
+        <v>0.98</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -565,16 +565,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="D5" t="n">
-        <v>2.27</v>
+        <v>7.4</v>
       </c>
       <c r="E5" t="n">
-        <v>98.36</v>
+        <v>95.45</v>
       </c>
       <c r="F5" t="n">
-        <v>0.42</v>
+        <v>0.6</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -598,13 +598,13 @@
         <v>0.12</v>
       </c>
       <c r="D6" t="n">
-        <v>1.64</v>
+        <v>4.55</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3</v>
+        <v>0.37</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>

</xml_diff>